<commit_message>
feat: add `has_curve` property and prioritize link selection logic
- Introduced `has_curve` attribute in `AggregatedValues` to track curve presence.
- Added `selection_priority` property to enhance sorting by curve presence and reference capacity.
- Updated link aggregation and selection logic to utilize the new `selection_priority`.
- Adjusted tests and expected output to reflect changes in link selection criteria.
</commit_message>
<xml_diff>
--- a/tests/antares/resources/expected_output_files/links/PEMMDB_LINK.xlsx
+++ b/tests/antares/resources/expected_output_files/links/PEMMDB_LINK.xlsx
@@ -1170,28 +1170,28 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>1500</v>
+        <v>1616</v>
       </c>
       <c r="C14" t="n">
-        <v>1674</v>
+        <v>1755</v>
       </c>
       <c r="D14" t="n">
-        <v>1500</v>
+        <v>1616</v>
       </c>
       <c r="E14" t="n">
-        <v>1674</v>
+        <v>1755</v>
       </c>
       <c r="F14" t="n">
-        <v>1500</v>
+        <v>1623</v>
       </c>
       <c r="G14" t="n">
-        <v>1674</v>
+        <v>1771</v>
       </c>
       <c r="H14" t="n">
-        <v>1500</v>
+        <v>1623</v>
       </c>
       <c r="I14" t="n">
-        <v>1674</v>
+        <v>1771</v>
       </c>
       <c r="J14" t="b">
         <v>0</v>
@@ -2096,7 +2096,7 @@
         <v>0.0888888888888888</v>
       </c>
       <c r="P31" t="n">
-        <v>0.02</v>
+        <v>0.0888888888888888</v>
       </c>
     </row>
     <row r="32">
@@ -3614,13 +3614,13 @@
         </is>
       </c>
       <c r="B61" t="n">
-        <v>300</v>
+        <v>150</v>
       </c>
       <c r="C61" t="n">
         <v>150</v>
       </c>
       <c r="D61" t="n">
-        <v>300</v>
+        <v>150</v>
       </c>
       <c r="E61" t="n">
         <v>150</v>
@@ -3773,13 +3773,13 @@
         <v>873</v>
       </c>
       <c r="C64" t="n">
-        <v>1440</v>
+        <v>1337</v>
       </c>
       <c r="D64" t="n">
         <v>873</v>
       </c>
       <c r="E64" t="n">
-        <v>1440</v>
+        <v>1337</v>
       </c>
       <c r="F64" t="n">
         <v>863</v>
@@ -4394,28 +4394,28 @@
         </is>
       </c>
       <c r="B76" t="n">
-        <v>1080</v>
+        <v>1260</v>
       </c>
       <c r="C76" t="n">
-        <v>1153</v>
+        <v>1353</v>
       </c>
       <c r="D76" t="n">
-        <v>1080</v>
+        <v>1280</v>
       </c>
       <c r="E76" t="n">
-        <v>1153</v>
+        <v>1241</v>
       </c>
       <c r="F76" t="n">
-        <v>1080</v>
+        <v>1220</v>
       </c>
       <c r="G76" t="n">
-        <v>1153</v>
+        <v>1134</v>
       </c>
       <c r="H76" t="n">
-        <v>1080</v>
+        <v>1245</v>
       </c>
       <c r="I76" t="n">
-        <v>1153</v>
+        <v>1094</v>
       </c>
       <c r="J76" t="b">
         <v>0</v>
@@ -4657,25 +4657,25 @@
         <v>440</v>
       </c>
       <c r="C81" t="n">
-        <v>1120</v>
+        <v>1140</v>
       </c>
       <c r="D81" t="n">
         <v>440</v>
       </c>
       <c r="E81" t="n">
-        <v>1120</v>
+        <v>1140</v>
       </c>
       <c r="F81" t="n">
         <v>440</v>
       </c>
       <c r="G81" t="n">
-        <v>1120</v>
+        <v>1140</v>
       </c>
       <c r="H81" t="n">
         <v>440</v>
       </c>
       <c r="I81" t="n">
-        <v>1120</v>
+        <v>1140</v>
       </c>
       <c r="J81" t="b">
         <v>0</v>
@@ -5333,25 +5333,25 @@
         <v>2024</v>
       </c>
       <c r="C94" t="n">
-        <v>1820</v>
+        <v>1843</v>
       </c>
       <c r="D94" t="n">
         <v>2024</v>
       </c>
       <c r="E94" t="n">
-        <v>1820</v>
+        <v>1843</v>
       </c>
       <c r="F94" t="n">
-        <v>2024</v>
+        <v>2013</v>
       </c>
       <c r="G94" t="n">
-        <v>1820</v>
+        <v>1826</v>
       </c>
       <c r="H94" t="n">
-        <v>2024</v>
+        <v>2013</v>
       </c>
       <c r="I94" t="n">
-        <v>1820</v>
+        <v>1826</v>
       </c>
       <c r="J94" t="b">
         <v>0</v>
@@ -6310,28 +6310,28 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>1500</v>
+        <v>1616</v>
       </c>
       <c r="C14" t="n">
-        <v>1674</v>
+        <v>1755</v>
       </c>
       <c r="D14" t="n">
-        <v>1500</v>
+        <v>1616</v>
       </c>
       <c r="E14" t="n">
-        <v>1674</v>
+        <v>1755</v>
       </c>
       <c r="F14" t="n">
-        <v>1500</v>
+        <v>1623</v>
       </c>
       <c r="G14" t="n">
-        <v>1674</v>
+        <v>1771</v>
       </c>
       <c r="H14" t="n">
-        <v>1500</v>
+        <v>1623</v>
       </c>
       <c r="I14" t="n">
-        <v>1674</v>
+        <v>1771</v>
       </c>
       <c r="J14" t="b">
         <v>0</v>
@@ -6842,13 +6842,13 @@
         <v>620</v>
       </c>
       <c r="F24" t="n">
-        <v>840</v>
+        <v>838</v>
       </c>
       <c r="G24" t="n">
         <v>620</v>
       </c>
       <c r="H24" t="n">
-        <v>840</v>
+        <v>838</v>
       </c>
       <c r="I24" t="n">
         <v>620</v>
@@ -7337,10 +7337,10 @@
         <v>2</v>
       </c>
       <c r="O33" t="n">
-        <v>0.02</v>
+        <v>0.0888888888888888</v>
       </c>
       <c r="P33" t="n">
-        <v>0.02</v>
+        <v>0.0888888888888888</v>
       </c>
     </row>
     <row r="34">
@@ -7392,7 +7392,7 @@
         <v>0.0888888888888888</v>
       </c>
       <c r="P34" t="n">
-        <v>0.02</v>
+        <v>0.0888888888888888</v>
       </c>
     </row>
     <row r="35">
@@ -8962,13 +8962,13 @@
         </is>
       </c>
       <c r="B65" t="n">
-        <v>300</v>
+        <v>150</v>
       </c>
       <c r="C65" t="n">
         <v>150</v>
       </c>
       <c r="D65" t="n">
-        <v>300</v>
+        <v>150</v>
       </c>
       <c r="E65" t="n">
         <v>150</v>
@@ -9121,13 +9121,13 @@
         <v>873</v>
       </c>
       <c r="C68" t="n">
-        <v>1440</v>
+        <v>1337</v>
       </c>
       <c r="D68" t="n">
         <v>873</v>
       </c>
       <c r="E68" t="n">
-        <v>1440</v>
+        <v>1337</v>
       </c>
       <c r="F68" t="n">
         <v>863</v>
@@ -9846,28 +9846,28 @@
         </is>
       </c>
       <c r="B82" t="n">
-        <v>1080</v>
+        <v>1260</v>
       </c>
       <c r="C82" t="n">
-        <v>1153</v>
+        <v>1353</v>
       </c>
       <c r="D82" t="n">
-        <v>1080</v>
+        <v>1280</v>
       </c>
       <c r="E82" t="n">
-        <v>1153</v>
+        <v>1241</v>
       </c>
       <c r="F82" t="n">
-        <v>1080</v>
+        <v>1220</v>
       </c>
       <c r="G82" t="n">
-        <v>1153</v>
+        <v>1134</v>
       </c>
       <c r="H82" t="n">
-        <v>1080</v>
+        <v>1245</v>
       </c>
       <c r="I82" t="n">
-        <v>1153</v>
+        <v>1094</v>
       </c>
       <c r="J82" t="b">
         <v>0</v>
@@ -10109,25 +10109,25 @@
         <v>440</v>
       </c>
       <c r="C87" t="n">
-        <v>1120</v>
+        <v>1140</v>
       </c>
       <c r="D87" t="n">
         <v>440</v>
       </c>
       <c r="E87" t="n">
-        <v>1120</v>
+        <v>1140</v>
       </c>
       <c r="F87" t="n">
         <v>440</v>
       </c>
       <c r="G87" t="n">
-        <v>1120</v>
+        <v>1140</v>
       </c>
       <c r="H87" t="n">
         <v>440</v>
       </c>
       <c r="I87" t="n">
-        <v>1120</v>
+        <v>1140</v>
       </c>
       <c r="J87" t="b">
         <v>0</v>
@@ -10785,25 +10785,25 @@
         <v>2024</v>
       </c>
       <c r="C100" t="n">
-        <v>1820</v>
+        <v>1843</v>
       </c>
       <c r="D100" t="n">
         <v>2024</v>
       </c>
       <c r="E100" t="n">
-        <v>1820</v>
+        <v>1843</v>
       </c>
       <c r="F100" t="n">
-        <v>2024</v>
+        <v>2013</v>
       </c>
       <c r="G100" t="n">
-        <v>1820</v>
+        <v>1826</v>
       </c>
       <c r="H100" t="n">
-        <v>2024</v>
+        <v>2013</v>
       </c>
       <c r="I100" t="n">
-        <v>1820</v>
+        <v>1826</v>
       </c>
       <c r="J100" t="b">
         <v>0</v>

</xml_diff>

<commit_message>
refactor(constants): update HVDC link constants for better naming consistency
- Updated HVDC constant names in `constants.py` to align with new naming conventions (`_MW_` and `_FO_Rate_`).
- Adjusted related test output files to reflect changes.
</commit_message>
<xml_diff>
--- a/tests/antares/resources/expected_output_files/links/PEMMDB_LINK.xlsx
+++ b/tests/antares/resources/expected_output_files/links/PEMMDB_LINK.xlsx
@@ -510,12 +510,12 @@
       </c>
       <c r="K1" t="inlineStr">
         <is>
-          <t>HVDC_Direct</t>
+          <t>HVDC_MW_direct</t>
         </is>
       </c>
       <c r="L1" t="inlineStr">
         <is>
-          <t>HVDC_Indirect</t>
+          <t>HVDC_MW_Indirect</t>
         </is>
       </c>
       <c r="M1" t="inlineStr">
@@ -530,12 +530,12 @@
       </c>
       <c r="O1" t="inlineStr">
         <is>
-          <t>HVDC_For_Direct</t>
+          <t>HVDC_FO_Rate_direct</t>
         </is>
       </c>
       <c r="P1" t="inlineStr">
         <is>
-          <t>HVDC_For_Indirect</t>
+          <t>HVDC_FO_Rate_indirect</t>
         </is>
       </c>
     </row>
@@ -5650,12 +5650,12 @@
       </c>
       <c r="K1" t="inlineStr">
         <is>
-          <t>HVDC_Direct</t>
+          <t>HVDC_MW_direct</t>
         </is>
       </c>
       <c r="L1" t="inlineStr">
         <is>
-          <t>HVDC_Indirect</t>
+          <t>HVDC_MW_Indirect</t>
         </is>
       </c>
       <c r="M1" t="inlineStr">
@@ -5670,12 +5670,12 @@
       </c>
       <c r="O1" t="inlineStr">
         <is>
-          <t>HVDC_For_Direct</t>
+          <t>HVDC_FO_Rate_direct</t>
         </is>
       </c>
       <c r="P1" t="inlineStr">
         <is>
-          <t>HVDC_For_Indirect</t>
+          <t>HVDC_FO_Rate_indirect</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: add `mean_strict_positive` utility and improve HVDC aggregation logic
- Introduced `mean_strict_positive` utility function to compute the mean of strictly positive values.
- Updated HVDC aggregation logic in `parsing.py` to use `mean_strict_positive` for `hvdc_for`.
- Adjusted expected output file to reflect changes in aggregation calculations.
</commit_message>
<xml_diff>
--- a/tests/antares/resources/expected_output_files/links/PEMMDB_LINK.xlsx
+++ b/tests/antares/resources/expected_output_files/links/PEMMDB_LINK.xlsx
@@ -5525,7 +5525,7 @@
         <v>2</v>
       </c>
       <c r="O97" t="n">
-        <v>0.005</v>
+        <v>0.01</v>
       </c>
       <c r="P97" t="n">
         <v>0.01</v>
@@ -10977,7 +10977,7 @@
         <v>2</v>
       </c>
       <c r="O103" t="n">
-        <v>0.005</v>
+        <v>0.01</v>
       </c>
       <c r="P103" t="n">
         <v>0.01</v>

</xml_diff>

<commit_message>
refactor(parsing): remove unused `discrim_profil` logic and cleanup comments
- Eliminated the commented-out `discrim_profil` function to declutter code.
- Removed redundant test variable and outdated comments for clearer implementation.
</commit_message>
<xml_diff>
--- a/tests/antares/resources/expected_output_files/links/PEMMDB_LINK.xlsx
+++ b/tests/antares/resources/expected_output_files/links/PEMMDB_LINK.xlsx
@@ -1261,10 +1261,10 @@
         <v>1</v>
       </c>
       <c r="O15" t="n">
-        <v>0.06</v>
+        <v>0.02</v>
       </c>
       <c r="P15" t="n">
-        <v>0.06</v>
+        <v>0.02</v>
       </c>
     </row>
     <row r="16">
@@ -2873,10 +2873,10 @@
         <v>2</v>
       </c>
       <c r="O46" t="n">
-        <v>0.11</v>
+        <v>0.03</v>
       </c>
       <c r="P46" t="n">
-        <v>0.11</v>
+        <v>0.03</v>
       </c>
     </row>
     <row r="47">
@@ -3231,16 +3231,16 @@
         <v>700</v>
       </c>
       <c r="M53" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N53" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O53" t="n">
-        <v>0</v>
+        <v>0.08400000000000001</v>
       </c>
       <c r="P53" t="n">
-        <v>0</v>
+        <v>0.08400000000000001</v>
       </c>
     </row>
     <row r="54">
@@ -3340,12 +3340,8 @@
       <c r="N55" t="n">
         <v>2</v>
       </c>
-      <c r="O55" t="n">
-        <v>0</v>
-      </c>
-      <c r="P55" t="n">
-        <v>0</v>
-      </c>
+      <c r="O55" t="inlineStr"/>
+      <c r="P55" t="inlineStr"/>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
@@ -4531,16 +4527,16 @@
         <v>700</v>
       </c>
       <c r="M78" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N78" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O78" t="n">
-        <v>0.1</v>
+        <v>0.035</v>
       </c>
       <c r="P78" t="n">
-        <v>0.1</v>
+        <v>0.035</v>
       </c>
     </row>
     <row r="79">
@@ -6349,10 +6345,10 @@
         <v>1</v>
       </c>
       <c r="O16" t="n">
-        <v>0.06</v>
+        <v>0.02</v>
       </c>
       <c r="P16" t="n">
-        <v>0.06</v>
+        <v>0.02</v>
       </c>
     </row>
     <row r="17">
@@ -8117,10 +8113,10 @@
         <v>3</v>
       </c>
       <c r="O50" t="n">
-        <v>0.11</v>
+        <v>0.03</v>
       </c>
       <c r="P50" t="n">
-        <v>0.11</v>
+        <v>0.03</v>
       </c>
     </row>
     <row r="51">
@@ -8325,10 +8321,10 @@
         <v>1</v>
       </c>
       <c r="O54" t="n">
-        <v>0.03</v>
+        <v>0</v>
       </c>
       <c r="P54" t="n">
-        <v>0.03</v>
+        <v>0</v>
       </c>
     </row>
     <row r="55">
@@ -8475,16 +8471,16 @@
         <v>700</v>
       </c>
       <c r="M57" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N57" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O57" t="n">
-        <v>0</v>
+        <v>0.08400000000000001</v>
       </c>
       <c r="P57" t="n">
-        <v>0</v>
+        <v>0.08400000000000001</v>
       </c>
     </row>
     <row r="58">
@@ -8584,12 +8580,8 @@
       <c r="N59" t="n">
         <v>2</v>
       </c>
-      <c r="O59" t="n">
-        <v>0</v>
-      </c>
-      <c r="P59" t="n">
-        <v>0</v>
-      </c>
+      <c r="O59" t="inlineStr"/>
+      <c r="P59" t="inlineStr"/>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
@@ -9879,16 +9871,16 @@
         <v>700</v>
       </c>
       <c r="M84" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N84" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O84" t="n">
-        <v>0.1</v>
+        <v>0.035</v>
       </c>
       <c r="P84" t="n">
-        <v>0.1</v>
+        <v>0.035</v>
       </c>
     </row>
     <row r="85">

</xml_diff>

<commit_message>
refactor(links): simplify constants handling and improve parameter export
- Replaced hardcoded Hurdle Costs constants with a `DEFAULT_LINK_PARAMETERS` DataFrame for more flexible handling.
- Updated links parsing logic to use the new DataFrame for parameter export.
- Removed print statement from `get_peak_hour_label` in `MainParams`.
- Updated `PEMMDB_LINK.xlsx` in expected output files.
</commit_message>
<xml_diff>
--- a/tests/antares/resources/expected_output_files/links/PEMMDB_LINK.xlsx
+++ b/tests/antares/resources/expected_output_files/links/PEMMDB_LINK.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C2"/>
+  <dimension ref="A1:C3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -441,6 +441,19 @@
       </c>
       <c r="C2" t="n">
         <v>0.5</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>HVDC</t>
+        </is>
+      </c>
+      <c r="B3" t="b">
+        <v>0</v>
+      </c>
+      <c r="C3" t="b">
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: add rounding to "FOR" column in "Transfer Links.csv" and update related constants and parsing logic
</commit_message>
<xml_diff>
--- a/tests/antares/resources/expected_output_files/links/PEMMDB_LINK.xlsx
+++ b/tests/antares/resources/expected_output_files/links/PEMMDB_LINK.xlsx
@@ -1170,10 +1170,10 @@
         <v>1</v>
       </c>
       <c r="O13" t="n">
-        <v>0.0888888888888888</v>
+        <v>0.09</v>
       </c>
       <c r="P13" t="n">
-        <v>0.0888888888888888</v>
+        <v>0.09</v>
       </c>
     </row>
     <row r="14">
@@ -1586,10 +1586,10 @@
         <v>1</v>
       </c>
       <c r="O21" t="n">
-        <v>0.0888888888888888</v>
+        <v>0.09</v>
       </c>
       <c r="P21" t="n">
-        <v>0.0888888888888888</v>
+        <v>0.09</v>
       </c>
     </row>
     <row r="22">
@@ -1690,10 +1690,10 @@
         <v>1</v>
       </c>
       <c r="O23" t="n">
-        <v>0.0888888888888888</v>
+        <v>0.09</v>
       </c>
       <c r="P23" t="n">
-        <v>0.0888888888888888</v>
+        <v>0.09</v>
       </c>
     </row>
     <row r="24">
@@ -1742,10 +1742,10 @@
         <v>4</v>
       </c>
       <c r="O24" t="n">
-        <v>0.0888888888888888</v>
+        <v>0.09</v>
       </c>
       <c r="P24" t="n">
-        <v>0.0888888888888888</v>
+        <v>0.09</v>
       </c>
     </row>
     <row r="25">
@@ -1794,10 +1794,10 @@
         <v>2</v>
       </c>
       <c r="O25" t="n">
-        <v>0.0888888888888888</v>
+        <v>0.09</v>
       </c>
       <c r="P25" t="n">
-        <v>0.0888888888888888</v>
+        <v>0.09</v>
       </c>
     </row>
     <row r="26">
@@ -1846,10 +1846,10 @@
         <v>2</v>
       </c>
       <c r="O26" t="n">
-        <v>0.0888888888888888</v>
+        <v>0.09</v>
       </c>
       <c r="P26" t="n">
-        <v>0.0888888888888888</v>
+        <v>0.09</v>
       </c>
     </row>
     <row r="27">
@@ -1950,10 +1950,10 @@
         <v>2</v>
       </c>
       <c r="O28" t="n">
-        <v>0.08400000000000001</v>
+        <v>0.08</v>
       </c>
       <c r="P28" t="n">
-        <v>0.08400000000000001</v>
+        <v>0.08</v>
       </c>
     </row>
     <row r="29">
@@ -2158,10 +2158,10 @@
         <v>2</v>
       </c>
       <c r="O32" t="n">
-        <v>0.063</v>
+        <v>0.06</v>
       </c>
       <c r="P32" t="n">
-        <v>0.063</v>
+        <v>0.06</v>
       </c>
     </row>
     <row r="33">
@@ -2418,10 +2418,10 @@
         <v>2</v>
       </c>
       <c r="O37" t="n">
-        <v>0.012</v>
+        <v>0.01</v>
       </c>
       <c r="P37" t="n">
-        <v>0.012</v>
+        <v>0.01</v>
       </c>
     </row>
     <row r="38">
@@ -3042,10 +3042,10 @@
         <v>2</v>
       </c>
       <c r="O49" t="n">
-        <v>0.08400000000000001</v>
+        <v>0.08</v>
       </c>
       <c r="P49" t="n">
-        <v>0.08400000000000001</v>
+        <v>0.08</v>
       </c>
     </row>
   </sheetData>
@@ -3762,10 +3762,10 @@
         <v>1</v>
       </c>
       <c r="O13" t="n">
-        <v>0.0888888888888888</v>
+        <v>0.09</v>
       </c>
       <c r="P13" t="n">
-        <v>0.0888888888888888</v>
+        <v>0.09</v>
       </c>
     </row>
     <row r="14">
@@ -4178,10 +4178,10 @@
         <v>1</v>
       </c>
       <c r="O21" t="n">
-        <v>0.0888888888888888</v>
+        <v>0.09</v>
       </c>
       <c r="P21" t="n">
-        <v>0.0888888888888888</v>
+        <v>0.09</v>
       </c>
     </row>
     <row r="22">
@@ -4282,10 +4282,10 @@
         <v>1</v>
       </c>
       <c r="O23" t="n">
-        <v>0.0888888888888888</v>
+        <v>0.09</v>
       </c>
       <c r="P23" t="n">
-        <v>0.0888888888888888</v>
+        <v>0.09</v>
       </c>
     </row>
     <row r="24">
@@ -4334,10 +4334,10 @@
         <v>4</v>
       </c>
       <c r="O24" t="n">
-        <v>0.0888888888888888</v>
+        <v>0.09</v>
       </c>
       <c r="P24" t="n">
-        <v>0.0888888888888888</v>
+        <v>0.09</v>
       </c>
     </row>
     <row r="25">
@@ -4386,10 +4386,10 @@
         <v>2</v>
       </c>
       <c r="O25" t="n">
-        <v>0.0888888888888888</v>
+        <v>0.09</v>
       </c>
       <c r="P25" t="n">
-        <v>0.0888888888888888</v>
+        <v>0.09</v>
       </c>
     </row>
     <row r="26">
@@ -4438,10 +4438,10 @@
         <v>2</v>
       </c>
       <c r="O26" t="n">
-        <v>0.0888888888888888</v>
+        <v>0.09</v>
       </c>
       <c r="P26" t="n">
-        <v>0.0888888888888888</v>
+        <v>0.09</v>
       </c>
     </row>
     <row r="27">
@@ -4542,10 +4542,10 @@
         <v>2</v>
       </c>
       <c r="O28" t="n">
-        <v>0.08400000000000001</v>
+        <v>0.08</v>
       </c>
       <c r="P28" t="n">
-        <v>0.08400000000000001</v>
+        <v>0.08</v>
       </c>
     </row>
     <row r="29">
@@ -4750,10 +4750,10 @@
         <v>2</v>
       </c>
       <c r="O32" t="n">
-        <v>0.063</v>
+        <v>0.06</v>
       </c>
       <c r="P32" t="n">
-        <v>0.063</v>
+        <v>0.06</v>
       </c>
     </row>
     <row r="33">
@@ -4854,10 +4854,10 @@
         <v>2</v>
       </c>
       <c r="O34" t="n">
-        <v>0.064</v>
+        <v>0.06</v>
       </c>
       <c r="P34" t="n">
-        <v>0.064</v>
+        <v>0.06</v>
       </c>
     </row>
     <row r="35">
@@ -5010,10 +5010,10 @@
         <v>2</v>
       </c>
       <c r="O37" t="n">
-        <v>0.074</v>
+        <v>0.07000000000000001</v>
       </c>
       <c r="P37" t="n">
-        <v>0.074</v>
+        <v>0.07000000000000001</v>
       </c>
     </row>
     <row r="38">
@@ -5114,10 +5114,10 @@
         <v>4</v>
       </c>
       <c r="O39" t="n">
-        <v>0.036</v>
+        <v>0.035</v>
       </c>
       <c r="P39" t="n">
-        <v>0.036</v>
+        <v>0.035</v>
       </c>
     </row>
     <row r="40">
@@ -5738,10 +5738,10 @@
         <v>2</v>
       </c>
       <c r="O51" t="n">
-        <v>0.08400000000000001</v>
+        <v>0.08</v>
       </c>
       <c r="P51" t="n">
-        <v>0.08400000000000001</v>
+        <v>0.08</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
LINKS : Column FOR (#74)
* feat: add default fill value for "FOR" column in "Transfer Links.csv" and update related parsing logic

* feat: add rounding to "FOR" column in "Transfer Links.csv" and update related constants and parsing logic
</commit_message>
<xml_diff>
--- a/tests/antares/resources/expected_output_files/links/PEMMDB_LINK.xlsx
+++ b/tests/antares/resources/expected_output_files/links/PEMMDB_LINK.xlsx
@@ -1170,10 +1170,10 @@
         <v>1</v>
       </c>
       <c r="O13" t="n">
-        <v>0.0888888888888888</v>
+        <v>0.09</v>
       </c>
       <c r="P13" t="n">
-        <v>0.0888888888888888</v>
+        <v>0.09</v>
       </c>
     </row>
     <row r="14">
@@ -1586,10 +1586,10 @@
         <v>1</v>
       </c>
       <c r="O21" t="n">
-        <v>0.0888888888888888</v>
+        <v>0.09</v>
       </c>
       <c r="P21" t="n">
-        <v>0.0888888888888888</v>
+        <v>0.09</v>
       </c>
     </row>
     <row r="22">
@@ -1690,10 +1690,10 @@
         <v>1</v>
       </c>
       <c r="O23" t="n">
-        <v>0.0888888888888888</v>
+        <v>0.09</v>
       </c>
       <c r="P23" t="n">
-        <v>0.0888888888888888</v>
+        <v>0.09</v>
       </c>
     </row>
     <row r="24">
@@ -1742,10 +1742,10 @@
         <v>4</v>
       </c>
       <c r="O24" t="n">
-        <v>0.0888888888888888</v>
+        <v>0.09</v>
       </c>
       <c r="P24" t="n">
-        <v>0.0888888888888888</v>
+        <v>0.09</v>
       </c>
     </row>
     <row r="25">
@@ -1794,10 +1794,10 @@
         <v>2</v>
       </c>
       <c r="O25" t="n">
-        <v>0.0888888888888888</v>
+        <v>0.09</v>
       </c>
       <c r="P25" t="n">
-        <v>0.0888888888888888</v>
+        <v>0.09</v>
       </c>
     </row>
     <row r="26">
@@ -1846,10 +1846,10 @@
         <v>2</v>
       </c>
       <c r="O26" t="n">
-        <v>0.0888888888888888</v>
+        <v>0.09</v>
       </c>
       <c r="P26" t="n">
-        <v>0.0888888888888888</v>
+        <v>0.09</v>
       </c>
     </row>
     <row r="27">
@@ -1950,10 +1950,10 @@
         <v>2</v>
       </c>
       <c r="O28" t="n">
-        <v>0.08400000000000001</v>
+        <v>0.08</v>
       </c>
       <c r="P28" t="n">
-        <v>0.08400000000000001</v>
+        <v>0.08</v>
       </c>
     </row>
     <row r="29">
@@ -2158,10 +2158,10 @@
         <v>2</v>
       </c>
       <c r="O32" t="n">
-        <v>0.063</v>
+        <v>0.06</v>
       </c>
       <c r="P32" t="n">
-        <v>0.063</v>
+        <v>0.06</v>
       </c>
     </row>
     <row r="33">
@@ -2418,10 +2418,10 @@
         <v>2</v>
       </c>
       <c r="O37" t="n">
-        <v>0.012</v>
+        <v>0.01</v>
       </c>
       <c r="P37" t="n">
-        <v>0.012</v>
+        <v>0.01</v>
       </c>
     </row>
     <row r="38">
@@ -3042,10 +3042,10 @@
         <v>2</v>
       </c>
       <c r="O49" t="n">
-        <v>0.08400000000000001</v>
+        <v>0.08</v>
       </c>
       <c r="P49" t="n">
-        <v>0.08400000000000001</v>
+        <v>0.08</v>
       </c>
     </row>
   </sheetData>
@@ -3762,10 +3762,10 @@
         <v>1</v>
       </c>
       <c r="O13" t="n">
-        <v>0.0888888888888888</v>
+        <v>0.09</v>
       </c>
       <c r="P13" t="n">
-        <v>0.0888888888888888</v>
+        <v>0.09</v>
       </c>
     </row>
     <row r="14">
@@ -4178,10 +4178,10 @@
         <v>1</v>
       </c>
       <c r="O21" t="n">
-        <v>0.0888888888888888</v>
+        <v>0.09</v>
       </c>
       <c r="P21" t="n">
-        <v>0.0888888888888888</v>
+        <v>0.09</v>
       </c>
     </row>
     <row r="22">
@@ -4282,10 +4282,10 @@
         <v>1</v>
       </c>
       <c r="O23" t="n">
-        <v>0.0888888888888888</v>
+        <v>0.09</v>
       </c>
       <c r="P23" t="n">
-        <v>0.0888888888888888</v>
+        <v>0.09</v>
       </c>
     </row>
     <row r="24">
@@ -4334,10 +4334,10 @@
         <v>4</v>
       </c>
       <c r="O24" t="n">
-        <v>0.0888888888888888</v>
+        <v>0.09</v>
       </c>
       <c r="P24" t="n">
-        <v>0.0888888888888888</v>
+        <v>0.09</v>
       </c>
     </row>
     <row r="25">
@@ -4386,10 +4386,10 @@
         <v>2</v>
       </c>
       <c r="O25" t="n">
-        <v>0.0888888888888888</v>
+        <v>0.09</v>
       </c>
       <c r="P25" t="n">
-        <v>0.0888888888888888</v>
+        <v>0.09</v>
       </c>
     </row>
     <row r="26">
@@ -4438,10 +4438,10 @@
         <v>2</v>
       </c>
       <c r="O26" t="n">
-        <v>0.0888888888888888</v>
+        <v>0.09</v>
       </c>
       <c r="P26" t="n">
-        <v>0.0888888888888888</v>
+        <v>0.09</v>
       </c>
     </row>
     <row r="27">
@@ -4542,10 +4542,10 @@
         <v>2</v>
       </c>
       <c r="O28" t="n">
-        <v>0.08400000000000001</v>
+        <v>0.08</v>
       </c>
       <c r="P28" t="n">
-        <v>0.08400000000000001</v>
+        <v>0.08</v>
       </c>
     </row>
     <row r="29">
@@ -4750,10 +4750,10 @@
         <v>2</v>
       </c>
       <c r="O32" t="n">
-        <v>0.063</v>
+        <v>0.06</v>
       </c>
       <c r="P32" t="n">
-        <v>0.063</v>
+        <v>0.06</v>
       </c>
     </row>
     <row r="33">
@@ -4854,10 +4854,10 @@
         <v>2</v>
       </c>
       <c r="O34" t="n">
-        <v>0.064</v>
+        <v>0.06</v>
       </c>
       <c r="P34" t="n">
-        <v>0.064</v>
+        <v>0.06</v>
       </c>
     </row>
     <row r="35">
@@ -5010,10 +5010,10 @@
         <v>2</v>
       </c>
       <c r="O37" t="n">
-        <v>0.074</v>
+        <v>0.07000000000000001</v>
       </c>
       <c r="P37" t="n">
-        <v>0.074</v>
+        <v>0.07000000000000001</v>
       </c>
     </row>
     <row r="38">
@@ -5114,10 +5114,10 @@
         <v>4</v>
       </c>
       <c r="O39" t="n">
-        <v>0.036</v>
+        <v>0.035</v>
       </c>
       <c r="P39" t="n">
-        <v>0.036</v>
+        <v>0.035</v>
       </c>
     </row>
     <row r="40">
@@ -5738,10 +5738,10 @@
         <v>2</v>
       </c>
       <c r="O51" t="n">
-        <v>0.08400000000000001</v>
+        <v>0.08</v>
       </c>
       <c r="P51" t="n">
-        <v>0.08400000000000001</v>
+        <v>0.08</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
fix(constants): adjust default 'Hurdle Costs' value in `DEFAULT_LINK_PARAMETERS` and update related test artifact
</commit_message>
<xml_diff>
--- a/tests/antares/resources/expected_output_files/links/PEMMDB_LINK.xlsx
+++ b/tests/antares/resources/expected_output_files/links/PEMMDB_LINK.xlsx
@@ -437,10 +437,10 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>0.5</v>
+        <v>0.1</v>
       </c>
       <c r="C2" t="n">
-        <v>0.5</v>
+        <v>0.1</v>
       </c>
     </row>
     <row r="3">

</xml_diff>

<commit_message>
fix(constants): adjust default 'Hurdle Costs' value in `DEFAULT_LINK_PARAMETERS` and update related test artifact (#76)
</commit_message>
<xml_diff>
--- a/tests/antares/resources/expected_output_files/links/PEMMDB_LINK.xlsx
+++ b/tests/antares/resources/expected_output_files/links/PEMMDB_LINK.xlsx
@@ -437,10 +437,10 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>0.5</v>
+        <v>0.1</v>
       </c>
       <c r="C2" t="n">
-        <v>0.5</v>
+        <v>0.1</v>
       </c>
     </row>
     <row r="3">

</xml_diff>